<commit_message>
Fix the tab that shipped empty in the file we hand customers
Listing the one-file workbook's tabs to answer "which file do I send"
showed the handoff tab with one row where twelve rules should be. The
one-file build carried its own copy of the row-seeding logic, so when
handoff.xlsx gained seeded content the copy kept writing a single example
row -- and the file about to reach a customer was the broken one.

The duplication is the actual defect, so the two builds now share one
helper rather than agreeing by coincidence. Two tests pin the tab's
contents, which is what would have caught this without me counting rows
by hand.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018jnyT7GXAudGv2xRF1qQGc
</commit_message>
<xml_diff>
--- a/templates/lavabo-intake-onefile.xlsx
+++ b/templates/lavabo-intake-onefile.xlsx
@@ -9584,7 +9584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -9628,28 +9628,244 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Khách hỏi mẫu shop không bán</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Bên mình có bồn tắm massage không?</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Hỏi giá mẫu không có trong bảng giá</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
         <is>
           <t>chuyển ngay cho nhân viên</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>chị Hương</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr"/>
-      <c r="F2" s="4" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Mặc cả, xin giảm giá, xin giá sỉ</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>chuyển ngay cho nhân viên</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Tính tổng tiền nhiều món, giá combo</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>chuyển ngay cho nhân viên</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Đơn đã đặt: kiểm tra, sửa, hủy, giục giao</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>chuyển ngay cho nhân viên</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Khiếu nại, hàng lỗi, hàng vỡ</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>chuyển ngay cho nhân viên</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Yêu cầu bảo hành cụ thể</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>chuyển ngay cho nhân viên</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Khách gửi ảnh hàng bị lỗi</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>chuyển ngay cho nhân viên</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Mua sỉ, làm đại lý</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>chuyển ngay cho nhân viên</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Xuất hóa đơn VAT, hợp đồng, công nợ</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>chuyển ngay cho nhân viên</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Khách xin số tài khoản để chuyển tiền</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>chuyển ngay cho nhân viên</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Khách nói muốn gặp người thật</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>chuyển ngay cho nhân viên</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Khách tỏ ra khó chịu, bực bội</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>chuyển ngay cho nhân viên</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>có</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>